<commit_message>
2026-06-17 17:48 - snapshot
</commit_message>
<xml_diff>
--- a/job-listings-template.xlsx
+++ b/job-listings-template.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,17 +499,22 @@
           <t>Date Found</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Posted Date</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Job Description</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>Skip Reason</t>
         </is>

</xml_diff>